<commit_message>
Show the column-order note on the in-season page; sweep stale docs
`columnOrderNote()` now excludes a *final* end-of-season page rather than
the type: the in-season page's columns are the current draft's order, so it
carries the same sentence as the post-draft page beside it until the capture
that seals the file drops it. The "months gone" reasoning is kept and
narrowed to the final page.

Docs: RUNBOOK's "Open after the 2026 draft" keeper-flag section is rewritten
as settled (Sleeper slots keepers nowhere; they come off `roster.keepers`
with `keeperTier` stamped), its calendar echo removed, the automation
section now describes the Sep-Jan in-season capture step and all three
guards `--force` overrides, and the hero-card sequence in CLAUDE.md and
site-design.md runs through In-Season and End-of-Season.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/2026/rosters-end-of-season-2026-ffl.xlsx
+++ b/output/2026/rosters-end-of-season-2026-ffl.xlsx
@@ -189,7 +189,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="26" customWidth="1"/>
@@ -1254,6 +1254,13 @@
     <row r="28"/>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Column order is the 2026 draft order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Data retrieved Sep 3, 2026, 8:09 AM PT</t>
         </is>

</xml_diff>